<commit_message>
Update generated Nifty 50 workbook
</commit_message>
<xml_diff>
--- a/output/nifty50.xlsx
+++ b/output/nifty50.xlsx
@@ -536,22 +536,22 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1310.2</v>
+        <v>1304</v>
       </c>
       <c r="E2" t="n">
-        <v>1306.9594</v>
+        <v>1304.9889</v>
       </c>
       <c r="F2" t="n">
-        <v>54.0234</v>
+        <v>49.9671</v>
       </c>
       <c r="G2" t="n">
-        <v>47.7012</v>
+        <v>45.8305</v>
       </c>
       <c r="H2" t="n">
-        <v>42.069</v>
+        <v>41.4303</v>
       </c>
       <c r="I2" t="n">
-        <v>45.6854</v>
+        <v>46.3225</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -571,7 +571,7 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:44+00:00</t>
+          <t>2026-07-04T00:36:28+00:00</t>
         </is>
       </c>
     </row>
@@ -592,22 +592,22 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>798.5</v>
+        <v>801.05</v>
       </c>
       <c r="E3" t="n">
-        <v>799.0638</v>
+        <v>802.9155</v>
       </c>
       <c r="F3" t="n">
-        <v>52.9117</v>
+        <v>54.8354</v>
       </c>
       <c r="G3" t="n">
-        <v>60.1566</v>
+        <v>61.0127</v>
       </c>
       <c r="H3" t="n">
-        <v>43.5252</v>
+        <v>44.159</v>
       </c>
       <c r="I3" t="n">
-        <v>43.8177</v>
+        <v>44.1455</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -627,7 +627,7 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:44+00:00</t>
+          <t>2026-07-04T00:36:28+00:00</t>
         </is>
       </c>
     </row>
@@ -648,22 +648,22 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1874.4</v>
+        <v>1910.4</v>
       </c>
       <c r="E4" t="n">
-        <v>1872.5598</v>
+        <v>1904.581</v>
       </c>
       <c r="F4" t="n">
-        <v>55.1625</v>
+        <v>66.9118</v>
       </c>
       <c r="G4" t="n">
-        <v>54.7191</v>
+        <v>61.5939</v>
       </c>
       <c r="H4" t="n">
-        <v>48.8691</v>
+        <v>51.6248</v>
       </c>
       <c r="I4" t="n">
-        <v>57.598</v>
+        <v>60.1015</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -683,7 +683,7 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:45+00:00</t>
+          <t>2026-07-04T00:36:29+00:00</t>
         </is>
       </c>
     </row>
@@ -704,22 +704,22 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1379.6</v>
+        <v>1411.4</v>
       </c>
       <c r="E5" t="n">
-        <v>1376.5483</v>
+        <v>1412.4659</v>
       </c>
       <c r="F5" t="n">
-        <v>51.5049</v>
+        <v>72.3051</v>
       </c>
       <c r="G5" t="n">
-        <v>66.8533</v>
+        <v>72.8699</v>
       </c>
       <c r="H5" t="n">
-        <v>57.717</v>
+        <v>61.373</v>
       </c>
       <c r="I5" t="n">
-        <v>58.2809</v>
+        <v>60.4618</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -739,7 +739,7 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:45+00:00</t>
+          <t>2026-07-04T00:36:29+00:00</t>
         </is>
       </c>
     </row>
@@ -760,22 +760,22 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1041.1</v>
+        <v>1040</v>
       </c>
       <c r="E6" t="n">
-        <v>1035.6497</v>
+        <v>1042.2863</v>
       </c>
       <c r="F6" t="n">
-        <v>55.2711</v>
+        <v>47.7511</v>
       </c>
       <c r="G6" t="n">
-        <v>58.9642</v>
+        <v>56.7344</v>
       </c>
       <c r="H6" t="n">
-        <v>53.3898</v>
+        <v>53.226</v>
       </c>
       <c r="I6" t="n">
-        <v>58.8642</v>
+        <v>59.5108</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -795,7 +795,7 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:46+00:00</t>
+          <t>2026-07-04T00:36:30+00:00</t>
         </is>
       </c>
     </row>
@@ -816,22 +816,22 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2003</v>
+        <v>2093.5</v>
       </c>
       <c r="E7" t="n">
-        <v>2028.976</v>
+        <v>2098.6365</v>
       </c>
       <c r="F7" t="n">
-        <v>29.1443</v>
+        <v>56.8897</v>
       </c>
       <c r="G7" t="n">
-        <v>30.0902</v>
+        <v>43.4567</v>
       </c>
       <c r="H7" t="n">
-        <v>22.977</v>
+        <v>25.3472</v>
       </c>
       <c r="I7" t="n">
-        <v>28.3992</v>
+        <v>30.1424</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -851,7 +851,7 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:47+00:00</t>
+          <t>2026-07-04T00:36:31+00:00</t>
         </is>
       </c>
     </row>
@@ -872,22 +872,22 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1016</v>
+        <v>1031.4</v>
       </c>
       <c r="E8" t="n">
-        <v>1013.4245</v>
+        <v>1032.5573</v>
       </c>
       <c r="F8" t="n">
-        <v>68.9751</v>
+        <v>65.84950000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>71.56140000000001</v>
+        <v>74.3411</v>
       </c>
       <c r="H8" t="n">
-        <v>60.2364</v>
+        <v>61.7256</v>
       </c>
       <c r="I8" t="n">
-        <v>58.2679</v>
+        <v>59.5785</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -907,7 +907,7 @@
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:47+00:00</t>
+          <t>2026-07-04T00:36:31+00:00</t>
         </is>
       </c>
     </row>
@@ -928,22 +928,22 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>4089.1</v>
+        <v>4026.6</v>
       </c>
       <c r="E9" t="n">
-        <v>4108.5053</v>
+        <v>4043.8726</v>
       </c>
       <c r="F9" t="n">
-        <v>24.4369</v>
+        <v>33.6778</v>
       </c>
       <c r="G9" t="n">
-        <v>49.5399</v>
+        <v>43.4321</v>
       </c>
       <c r="H9" t="n">
-        <v>54.1386</v>
+        <v>52.0276</v>
       </c>
       <c r="I9" t="n">
-        <v>59.5835</v>
+        <v>56.9616</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -963,7 +963,7 @@
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:48+00:00</t>
+          <t>2026-07-04T00:36:32+00:00</t>
         </is>
       </c>
     </row>
@@ -984,22 +984,22 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2179</v>
+        <v>2201.2</v>
       </c>
       <c r="E10" t="n">
-        <v>2166.7421</v>
+        <v>2206.3708</v>
       </c>
       <c r="F10" t="n">
-        <v>59.6079</v>
+        <v>58.1393</v>
       </c>
       <c r="G10" t="n">
-        <v>51.1596</v>
+        <v>54.0816</v>
       </c>
       <c r="H10" t="n">
-        <v>44.6443</v>
+        <v>46.5215</v>
       </c>
       <c r="I10" t="n">
-        <v>42.0001</v>
+        <v>44.992</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1019,7 +1019,7 @@
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:49+00:00</t>
+          <t>2026-07-04T00:36:33+00:00</t>
         </is>
       </c>
     </row>
@@ -1040,22 +1040,22 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1872.8</v>
+        <v>1904.8</v>
       </c>
       <c r="E11" t="n">
-        <v>1873.6817</v>
+        <v>1908.5896</v>
       </c>
       <c r="F11" t="n">
-        <v>51.1248</v>
+        <v>62.1879</v>
       </c>
       <c r="G11" t="n">
-        <v>62.941</v>
+        <v>70.23390000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>60.2606</v>
+        <v>62.598</v>
       </c>
       <c r="I11" t="n">
-        <v>60.2125</v>
+        <v>61.7627</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -1075,7 +1075,7 @@
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:49+00:00</t>
+          <t>2026-07-04T00:36:33+00:00</t>
         </is>
       </c>
     </row>
@@ -1096,22 +1096,22 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>14341</v>
+        <v>14366</v>
       </c>
       <c r="E12" t="n">
-        <v>14332.5129</v>
+        <v>14424.9756</v>
       </c>
       <c r="F12" t="n">
-        <v>70.18389999999999</v>
+        <v>59.0494</v>
       </c>
       <c r="G12" t="n">
-        <v>66.8603</v>
+        <v>66.5433</v>
       </c>
       <c r="H12" t="n">
-        <v>55.097</v>
+        <v>55.3129</v>
       </c>
       <c r="I12" t="n">
-        <v>54.8393</v>
+        <v>55.889</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1131,7 +1131,7 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:50+00:00</t>
+          <t>2026-07-04T00:36:34+00:00</t>
         </is>
       </c>
     </row>
@@ -1152,22 +1152,22 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1374.6</v>
+        <v>1342.1</v>
       </c>
       <c r="E13" t="n">
-        <v>1368.6586</v>
+        <v>1353.0089</v>
       </c>
       <c r="F13" t="n">
-        <v>54.8852</v>
+        <v>34.2202</v>
       </c>
       <c r="G13" t="n">
-        <v>61.8307</v>
+        <v>51.4408</v>
       </c>
       <c r="H13" t="n">
-        <v>60.5319</v>
+        <v>56.0612</v>
       </c>
       <c r="I13" t="n">
-        <v>59.9114</v>
+        <v>59.6569</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1187,7 +1187,7 @@
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:50+00:00</t>
+          <t>2026-07-04T00:36:35+00:00</t>
         </is>
       </c>
     </row>
@@ -1208,22 +1208,22 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1859.1</v>
+        <v>1874.2</v>
       </c>
       <c r="E14" t="n">
-        <v>1853.3692</v>
+        <v>1876.0671</v>
       </c>
       <c r="F14" t="n">
-        <v>68.8622</v>
+        <v>58.7049</v>
       </c>
       <c r="G14" t="n">
-        <v>61.0874</v>
+        <v>62.2876</v>
       </c>
       <c r="H14" t="n">
-        <v>70.5258</v>
+        <v>71.26000000000001</v>
       </c>
       <c r="I14" t="n">
-        <v>66.7225</v>
+        <v>68.3135</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1243,7 +1243,7 @@
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:51+00:00</t>
+          <t>2026-07-04T00:36:35+00:00</t>
         </is>
       </c>
     </row>
@@ -1264,22 +1264,22 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>988.4</v>
+        <v>1047.2</v>
       </c>
       <c r="E15" t="n">
-        <v>998.5566</v>
+        <v>1049.8596</v>
       </c>
       <c r="F15" t="n">
-        <v>25.3952</v>
+        <v>61.4464</v>
       </c>
       <c r="G15" t="n">
-        <v>28.9757</v>
+        <v>41.9614</v>
       </c>
       <c r="H15" t="n">
-        <v>26.8772</v>
+        <v>30.1314</v>
       </c>
       <c r="I15" t="n">
-        <v>29.9983</v>
+        <v>32.7669</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1299,7 +1299,7 @@
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:52+00:00</t>
+          <t>2026-07-04T00:36:36+00:00</t>
         </is>
       </c>
     </row>
@@ -1320,22 +1320,22 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>3126.3</v>
+        <v>3212.1</v>
       </c>
       <c r="E16" t="n">
-        <v>3089.0518</v>
+        <v>3178.4963</v>
       </c>
       <c r="F16" t="n">
-        <v>73.47620000000001</v>
+        <v>67.71469999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>64.98739999999999</v>
+        <v>69.22329999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>72.9701</v>
+        <v>74.56610000000001</v>
       </c>
       <c r="I16" t="n">
-        <v>59.0492</v>
+        <v>61.2479</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1355,7 +1355,7 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:52+00:00</t>
+          <t>2026-07-04T00:36:36+00:00</t>
         </is>
       </c>
     </row>
@@ -1376,22 +1376,22 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>399.15</v>
+        <v>396.75</v>
       </c>
       <c r="E17" t="n">
-        <v>396.1266</v>
+        <v>396.9924</v>
       </c>
       <c r="F17" t="n">
-        <v>52.2709</v>
+        <v>45.5417</v>
       </c>
       <c r="G17" t="n">
-        <v>53.6604</v>
+        <v>51.0411</v>
       </c>
       <c r="H17" t="n">
-        <v>51.5913</v>
+        <v>50.6016</v>
       </c>
       <c r="I17" t="n">
-        <v>50.5056</v>
+        <v>51.4176</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1411,7 +1411,7 @@
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:53+00:00</t>
+          <t>2026-07-04T00:36:37+00:00</t>
         </is>
       </c>
     </row>
@@ -1432,22 +1432,22 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>4409.5</v>
+        <v>4461.1</v>
       </c>
       <c r="E18" t="n">
-        <v>4453.5089</v>
+        <v>4475.3838</v>
       </c>
       <c r="F18" t="n">
-        <v>59.1398</v>
+        <v>58.1427</v>
       </c>
       <c r="G18" t="n">
-        <v>60.6815</v>
+        <v>62.6287</v>
       </c>
       <c r="H18" t="n">
-        <v>57.2802</v>
+        <v>58.5507</v>
       </c>
       <c r="I18" t="n">
-        <v>61.2557</v>
+        <v>61.9381</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1467,7 +1467,7 @@
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:53+00:00</t>
+          <t>2026-07-04T00:36:38+00:00</t>
         </is>
       </c>
     </row>
@@ -1488,22 +1488,22 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3140.6</v>
+        <v>3136.9</v>
       </c>
       <c r="E19" t="n">
-        <v>3141.253</v>
+        <v>3148.1162</v>
       </c>
       <c r="F19" t="n">
-        <v>56.315</v>
+        <v>50.1785</v>
       </c>
       <c r="G19" t="n">
-        <v>54.2181</v>
+        <v>53.2359</v>
       </c>
       <c r="H19" t="n">
-        <v>46.8837</v>
+        <v>46.7475</v>
       </c>
       <c r="I19" t="n">
-        <v>54.2053</v>
+        <v>55.8025</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:54+00:00</t>
+          <t>2026-07-04T00:36:38+00:00</t>
         </is>
       </c>
     </row>
@@ -1544,22 +1544,22 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>290.65</v>
+        <v>289.95</v>
       </c>
       <c r="E20" t="n">
-        <v>289.4867</v>
+        <v>290.3776</v>
       </c>
       <c r="F20" t="n">
-        <v>56.3446</v>
+        <v>51.0846</v>
       </c>
       <c r="G20" t="n">
-        <v>49.7462</v>
+        <v>48.5242</v>
       </c>
       <c r="H20" t="n">
-        <v>36.3389</v>
+        <v>35.8912</v>
       </c>
       <c r="I20" t="n">
-        <v>32.3957</v>
+        <v>33.2313</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1579,7 +1579,7 @@
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:54+00:00</t>
+          <t>2026-07-04T00:36:39+00:00</t>
         </is>
       </c>
     </row>
@@ -1600,22 +1600,22 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>358.9</v>
+        <v>356.45</v>
       </c>
       <c r="E21" t="n">
-        <v>358.2264</v>
+        <v>357.9482</v>
       </c>
       <c r="F21" t="n">
-        <v>55.3907</v>
+        <v>45.6007</v>
       </c>
       <c r="G21" t="n">
-        <v>43.7279</v>
+        <v>41.1745</v>
       </c>
       <c r="H21" t="n">
-        <v>46.2453</v>
+        <v>45.1748</v>
       </c>
       <c r="I21" t="n">
-        <v>53.8857</v>
+        <v>53.8362</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:55+00:00</t>
+          <t>2026-07-04T00:36:40+00:00</t>
         </is>
       </c>
     </row>
@@ -1656,22 +1656,22 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>11453</v>
+        <v>11723</v>
       </c>
       <c r="E22" t="n">
-        <v>11417.209</v>
+        <v>11702.6809</v>
       </c>
       <c r="F22" t="n">
-        <v>56.644</v>
+        <v>74.09229999999999</v>
       </c>
       <c r="G22" t="n">
-        <v>53.3551</v>
+        <v>61.1607</v>
       </c>
       <c r="H22" t="n">
-        <v>47.8324</v>
+        <v>51.1967</v>
       </c>
       <c r="I22" t="n">
-        <v>50.6788</v>
+        <v>53.9388</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1691,7 +1691,7 @@
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:56+00:00</t>
+          <t>2026-07-04T00:36:40+00:00</t>
         </is>
       </c>
     </row>
@@ -1712,22 +1712,22 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>415.4</v>
+        <v>418.05</v>
       </c>
       <c r="E23" t="n">
-        <v>414.8098</v>
+        <v>420.5892</v>
       </c>
       <c r="F23" t="n">
-        <v>55.7903</v>
+        <v>54.6009</v>
       </c>
       <c r="G23" t="n">
-        <v>49.5364</v>
+        <v>51.8111</v>
       </c>
       <c r="H23" t="n">
-        <v>48.567</v>
+        <v>49.3582</v>
       </c>
       <c r="I23" t="n">
-        <v>60.9067</v>
+        <v>61.7207</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1747,7 +1747,7 @@
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:56+00:00</t>
+          <t>2026-07-04T00:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -1768,22 +1768,22 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1220</v>
+        <v>1230.2</v>
       </c>
       <c r="E24" t="n">
-        <v>1218.6566</v>
+        <v>1233.9481</v>
       </c>
       <c r="F24" t="n">
-        <v>37.221</v>
+        <v>53.5028</v>
       </c>
       <c r="G24" t="n">
-        <v>33.896</v>
+        <v>39.6509</v>
       </c>
       <c r="H24" t="n">
-        <v>49.6124</v>
+        <v>51.2107</v>
       </c>
       <c r="I24" t="n">
-        <v>61.2384</v>
+        <v>61.4456</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1803,7 +1803,7 @@
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:57+00:00</t>
+          <t>2026-07-04T00:36:41+00:00</t>
         </is>
       </c>
     </row>
@@ -1824,22 +1824,22 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>234.26</v>
+        <v>237.84</v>
       </c>
       <c r="E25" t="n">
-        <v>234.7174</v>
+        <v>238.0407</v>
       </c>
       <c r="F25" t="n">
-        <v>45.3057</v>
+        <v>57.3274</v>
       </c>
       <c r="G25" t="n">
-        <v>24.0158</v>
+        <v>30.8849</v>
       </c>
       <c r="H25" t="n">
-        <v>37.0241</v>
+        <v>38.8923</v>
       </c>
       <c r="I25" t="n">
-        <v>46.5337</v>
+        <v>47.2865</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -1859,7 +1859,7 @@
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:58+00:00</t>
+          <t>2026-07-04T00:36:42+00:00</t>
         </is>
       </c>
     </row>
@@ -1880,22 +1880,22 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1040.2</v>
+        <v>1139</v>
       </c>
       <c r="E26" t="n">
-        <v>1056.593</v>
+        <v>1138.2425</v>
       </c>
       <c r="F26" t="n">
-        <v>15.7653</v>
+        <v>69.42149999999999</v>
       </c>
       <c r="G26" t="n">
-        <v>26.4072</v>
+        <v>51.6208</v>
       </c>
       <c r="H26" t="n">
-        <v>26.1649</v>
+        <v>34.0994</v>
       </c>
       <c r="I26" t="n">
-        <v>35.3218</v>
+        <v>38.6402</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -1915,7 +1915,7 @@
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:58+00:00</t>
+          <t>2026-07-04T00:36:43+00:00</t>
         </is>
       </c>
     </row>
@@ -1936,22 +1936,22 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1794.6</v>
+        <v>1895.6</v>
       </c>
       <c r="E27" t="n">
-        <v>1768.383</v>
+        <v>1895.7804</v>
       </c>
       <c r="F27" t="n">
-        <v>62.6199</v>
+        <v>75.33410000000001</v>
       </c>
       <c r="G27" t="n">
-        <v>57.7032</v>
+        <v>70.8154</v>
       </c>
       <c r="H27" t="n">
-        <v>47.6114</v>
+        <v>54.3064</v>
       </c>
       <c r="I27" t="n">
-        <v>48.3807</v>
+        <v>53.0227</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -1971,7 +1971,7 @@
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:59+00:00</t>
+          <t>2026-07-04T00:36:43+00:00</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1992,22 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1450.7</v>
+        <v>1459.8</v>
       </c>
       <c r="E28" t="n">
-        <v>1442.63</v>
+        <v>1453.5648</v>
       </c>
       <c r="F28" t="n">
-        <v>68.12779999999999</v>
+        <v>63.6639</v>
       </c>
       <c r="G28" t="n">
-        <v>61.4893</v>
+        <v>62.4121</v>
       </c>
       <c r="H28" t="n">
-        <v>64.5107</v>
+        <v>65.304</v>
       </c>
       <c r="I28" t="n">
-        <v>59.851</v>
+        <v>62.3019</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -2027,7 +2027,7 @@
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-07-01T08:17:59+00:00</t>
+          <t>2026-07-04T00:36:44+00:00</t>
         </is>
       </c>
     </row>
@@ -2048,22 +2048,22 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>9844</v>
+        <v>9785.5</v>
       </c>
       <c r="E29" t="n">
-        <v>9841.6456</v>
+        <v>9819.8928</v>
       </c>
       <c r="F29" t="n">
-        <v>55.6858</v>
+        <v>47.6203</v>
       </c>
       <c r="G29" t="n">
-        <v>43.44</v>
+        <v>41.6791</v>
       </c>
       <c r="H29" t="n">
-        <v>51.6667</v>
+        <v>50.6935</v>
       </c>
       <c r="I29" t="n">
-        <v>57.1729</v>
+        <v>57.5961</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -2083,7 +2083,7 @@
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:00+00:00</t>
+          <t>2026-07-04T00:36:45+00:00</t>
         </is>
       </c>
     </row>
@@ -2104,22 +2104,22 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>434</v>
+        <v>438.7</v>
       </c>
       <c r="E30" t="n">
-        <v>436.3001</v>
+        <v>440.6804</v>
       </c>
       <c r="F30" t="n">
-        <v>35.6062</v>
+        <v>51.3482</v>
       </c>
       <c r="G30" t="n">
-        <v>37.0566</v>
+        <v>41.3718</v>
       </c>
       <c r="H30" t="n">
-        <v>48.2587</v>
+        <v>49.681</v>
       </c>
       <c r="I30" t="n">
-        <v>56.6069</v>
+        <v>56.5296</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -2139,7 +2139,7 @@
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:00+00:00</t>
+          <t>2026-07-04T00:36:45+00:00</t>
         </is>
       </c>
     </row>
@@ -2160,22 +2160,22 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>287.65</v>
+        <v>287.85</v>
       </c>
       <c r="E31" t="n">
-        <v>287.0648</v>
+        <v>289.4696</v>
       </c>
       <c r="F31" t="n">
-        <v>52.6438</v>
+        <v>49.2542</v>
       </c>
       <c r="G31" t="n">
-        <v>46.0857</v>
+        <v>46.5004</v>
       </c>
       <c r="H31" t="n">
-        <v>47.2624</v>
+        <v>47.3887</v>
       </c>
       <c r="I31" t="n">
-        <v>51.607</v>
+        <v>51.9704</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -2195,7 +2195,7 @@
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:01+00:00</t>
+          <t>2026-07-04T00:36:46+00:00</t>
         </is>
       </c>
     </row>
@@ -2216,22 +2216,22 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>277.1</v>
+        <v>281.65</v>
       </c>
       <c r="E32" t="n">
-        <v>272.7086</v>
+        <v>283.9016</v>
       </c>
       <c r="F32" t="n">
-        <v>86.13979999999999</v>
+        <v>65.08929999999999</v>
       </c>
       <c r="G32" t="n">
-        <v>69.0431</v>
+        <v>71.3334</v>
       </c>
       <c r="H32" t="n">
-        <v>56.2026</v>
+        <v>57.4636</v>
       </c>
       <c r="I32" t="n">
-        <v>55.3262</v>
+        <v>58.5815</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -2251,7 +2251,7 @@
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:01+00:00</t>
+          <t>2026-07-04T00:36:46+00:00</t>
         </is>
       </c>
     </row>
@@ -2272,22 +2272,22 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>2716.7</v>
+        <v>2737.8</v>
       </c>
       <c r="E33" t="n">
-        <v>2688.584</v>
+        <v>2742.5108</v>
       </c>
       <c r="F33" t="n">
-        <v>66.7346</v>
+        <v>59.3144</v>
       </c>
       <c r="G33" t="n">
-        <v>58.2127</v>
+        <v>60.3118</v>
       </c>
       <c r="H33" t="n">
-        <v>59.575</v>
+        <v>60.5324</v>
       </c>
       <c r="I33" t="n">
-        <v>50.9914</v>
+        <v>53.1762</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
@@ -2307,7 +2307,7 @@
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:02+00:00</t>
+          <t>2026-07-04T00:36:47+00:00</t>
         </is>
       </c>
     </row>
@@ -2328,22 +2328,22 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1048</v>
+        <v>1063.6</v>
       </c>
       <c r="E34" t="n">
-        <v>1050.55</v>
+        <v>1071.1931</v>
       </c>
       <c r="F34" t="n">
-        <v>59.9805</v>
+        <v>55.0519</v>
       </c>
       <c r="G34" t="n">
-        <v>69.11920000000001</v>
+        <v>71.244</v>
       </c>
       <c r="H34" t="n">
-        <v>60.6735</v>
+        <v>61.9226</v>
       </c>
       <c r="I34" t="n">
-        <v>67.5727</v>
+        <v>68.36839999999999</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
@@ -2363,7 +2363,7 @@
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:02+00:00</t>
+          <t>2026-07-04T00:36:48+00:00</t>
         </is>
       </c>
     </row>
@@ -2384,22 +2384,22 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>186.46</v>
+        <v>189.8</v>
       </c>
       <c r="E35" t="n">
-        <v>187.2886</v>
+        <v>191.19</v>
       </c>
       <c r="F35" t="n">
-        <v>32.8845</v>
+        <v>55.1582</v>
       </c>
       <c r="G35" t="n">
-        <v>26.0117</v>
+        <v>36.7315</v>
       </c>
       <c r="H35" t="n">
-        <v>42.7812</v>
+        <v>45.0421</v>
       </c>
       <c r="I35" t="n">
-        <v>56.126</v>
+        <v>56.6125</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
@@ -2419,7 +2419,7 @@
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:03+00:00</t>
+          <t>2026-07-04T00:36:49+00:00</t>
         </is>
       </c>
     </row>
@@ -2440,22 +2440,22 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>3135</v>
+        <v>3180.9</v>
       </c>
       <c r="E36" t="n">
-        <v>3128.6278</v>
+        <v>3198.1068</v>
       </c>
       <c r="F36" t="n">
-        <v>57.7495</v>
+        <v>62.2209</v>
       </c>
       <c r="G36" t="n">
-        <v>56.7032</v>
+        <v>62.6148</v>
       </c>
       <c r="H36" t="n">
-        <v>64.80840000000001</v>
+        <v>66.70180000000001</v>
       </c>
       <c r="I36" t="n">
-        <v>63.5302</v>
+        <v>65.18049999999999</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -2475,7 +2475,7 @@
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:04+00:00</t>
+          <t>2026-07-04T00:36:49+00:00</t>
         </is>
       </c>
     </row>
@@ -2496,22 +2496,22 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>941.05</v>
+        <v>953.2</v>
       </c>
       <c r="E37" t="n">
-        <v>945.6038</v>
+        <v>963.5848</v>
       </c>
       <c r="F37" t="n">
-        <v>30.756</v>
+        <v>46.7358</v>
       </c>
       <c r="G37" t="n">
-        <v>30.3309</v>
+        <v>34.9619</v>
       </c>
       <c r="H37" t="n">
-        <v>46.6623</v>
+        <v>48.039</v>
       </c>
       <c r="I37" t="n">
-        <v>60.515</v>
+        <v>60.2698</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -2531,7 +2531,7 @@
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:04+00:00</t>
+          <t>2026-07-04T00:36:50+00:00</t>
         </is>
       </c>
     </row>
@@ -2552,22 +2552,22 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>5375</v>
+        <v>5426.5</v>
       </c>
       <c r="E38" t="n">
-        <v>5365.5923</v>
+        <v>5425.1048</v>
       </c>
       <c r="F38" t="n">
-        <v>63.8475</v>
+        <v>58.3486</v>
       </c>
       <c r="G38" t="n">
-        <v>71.67659999999999</v>
+        <v>72.1606</v>
       </c>
       <c r="H38" t="n">
-        <v>62.6531</v>
+        <v>63.9871</v>
       </c>
       <c r="I38" t="n">
-        <v>58.5181</v>
+        <v>59.0351</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
@@ -2587,7 +2587,7 @@
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:05+00:00</t>
+          <t>2026-07-04T00:36:51+00:00</t>
         </is>
       </c>
     </row>
@@ -2608,22 +2608,22 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>7136</v>
+        <v>7339.5</v>
       </c>
       <c r="E39" t="n">
-        <v>7109.8381</v>
+        <v>7309.9664</v>
       </c>
       <c r="F39" t="n">
-        <v>36.3106</v>
+        <v>58.9928</v>
       </c>
       <c r="G39" t="n">
-        <v>40.9491</v>
+        <v>49.8811</v>
       </c>
       <c r="H39" t="n">
-        <v>49.6036</v>
+        <v>53.0347</v>
       </c>
       <c r="I39" t="n">
-        <v>61.8775</v>
+        <v>63.9682</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
@@ -2643,7 +2643,7 @@
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:05+00:00</t>
+          <t>2026-07-04T00:36:51+00:00</t>
         </is>
       </c>
     </row>
@@ -2664,22 +2664,22 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>170.15</v>
+        <v>176.08</v>
       </c>
       <c r="E40" t="n">
-        <v>170.4225</v>
+        <v>176.7024</v>
       </c>
       <c r="F40" t="n">
-        <v>30.9413</v>
+        <v>57.2853</v>
       </c>
       <c r="G40" t="n">
-        <v>27.0828</v>
+        <v>39.9129</v>
       </c>
       <c r="H40" t="n">
-        <v>28.6928</v>
+        <v>31.2911</v>
       </c>
       <c r="I40" t="n">
-        <v>34.4528</v>
+        <v>36.2938</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
@@ -2699,7 +2699,7 @@
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:06+00:00</t>
+          <t>2026-07-04T00:36:52+00:00</t>
         </is>
       </c>
     </row>
@@ -2720,22 +2720,22 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1786</v>
+        <v>1788.7</v>
       </c>
       <c r="E41" t="n">
-        <v>1768.5804</v>
+        <v>1787.4893</v>
       </c>
       <c r="F41" t="n">
-        <v>62.335</v>
+        <v>57.1577</v>
       </c>
       <c r="G41" t="n">
-        <v>49.76</v>
+        <v>50.3671</v>
       </c>
       <c r="H41" t="n">
-        <v>44.831</v>
+        <v>45.0289</v>
       </c>
       <c r="I41" t="n">
-        <v>51.9765</v>
+        <v>53.0919</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
@@ -2755,7 +2755,7 @@
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:07+00:00</t>
+          <t>2026-07-04T00:36:52+00:00</t>
         </is>
       </c>
     </row>
@@ -2776,22 +2776,22 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>3278.4</v>
+        <v>3340.6</v>
       </c>
       <c r="E42" t="n">
-        <v>3277.5471</v>
+        <v>3360.4029</v>
       </c>
       <c r="F42" t="n">
-        <v>55.6367</v>
+        <v>59.4535</v>
       </c>
       <c r="G42" t="n">
-        <v>72.27849999999999</v>
+        <v>75.4044</v>
       </c>
       <c r="H42" t="n">
-        <v>55.8932</v>
+        <v>57.3327</v>
       </c>
       <c r="I42" t="n">
-        <v>44.287</v>
+        <v>44.824</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
@@ -2811,7 +2811,7 @@
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:07+00:00</t>
+          <t>2026-07-04T00:36:53+00:00</t>
         </is>
       </c>
     </row>
@@ -2832,22 +2832,22 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>240.19</v>
+        <v>239.35</v>
       </c>
       <c r="E43" t="n">
-        <v>238.0545</v>
+        <v>240.194</v>
       </c>
       <c r="F43" t="n">
-        <v>61.4292</v>
+        <v>50.424</v>
       </c>
       <c r="G43" t="n">
-        <v>52.2939</v>
+        <v>50.9363</v>
       </c>
       <c r="H43" t="n">
-        <v>42.3625</v>
+        <v>41.7654</v>
       </c>
       <c r="I43" t="n">
-        <v>45.3712</v>
+        <v>45.9916</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
@@ -2867,7 +2867,7 @@
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:08+00:00</t>
+          <t>2026-07-04T00:36:54+00:00</t>
         </is>
       </c>
     </row>
@@ -2888,22 +2888,22 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>1358</v>
+        <v>1410.1</v>
       </c>
       <c r="E44" t="n">
-        <v>1368.2485</v>
+        <v>1424.5218</v>
       </c>
       <c r="F44" t="n">
-        <v>21.0244</v>
+        <v>47.4422</v>
       </c>
       <c r="G44" t="n">
-        <v>36.7843</v>
+        <v>45.9398</v>
       </c>
       <c r="H44" t="n">
-        <v>42.581</v>
+        <v>46.0504</v>
       </c>
       <c r="I44" t="n">
-        <v>47.8841</v>
+        <v>48.1194</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:08+00:00</t>
+          <t>2026-07-04T00:36:54+00:00</t>
         </is>
       </c>
     </row>
@@ -2944,22 +2944,22 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>347.05</v>
+        <v>344.1</v>
       </c>
       <c r="E45" t="n">
-        <v>349.8158</v>
+        <v>344.3171</v>
       </c>
       <c r="F45" t="n">
-        <v>39.4143</v>
+        <v>38.7045</v>
       </c>
       <c r="G45" t="n">
-        <v>39.1976</v>
+        <v>37.7482</v>
       </c>
       <c r="H45" t="n">
-        <v>41.4744</v>
+        <v>40.8707</v>
       </c>
       <c r="I45" t="n">
-        <v>36.8754</v>
+        <v>36.4686</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
@@ -2979,7 +2979,7 @@
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:09+00:00</t>
+          <t>2026-07-04T00:36:55+00:00</t>
         </is>
       </c>
     </row>
@@ -3000,22 +3000,22 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>8651</v>
+        <v>8893.5</v>
       </c>
       <c r="E46" t="n">
-        <v>8671.2817</v>
+        <v>8860.325800000001</v>
       </c>
       <c r="F46" t="n">
-        <v>51.7187</v>
+        <v>73.625</v>
       </c>
       <c r="G46" t="n">
-        <v>68.3439</v>
+        <v>75.5806</v>
       </c>
       <c r="H46" t="n">
-        <v>68.7364</v>
+        <v>71.9425</v>
       </c>
       <c r="I46" t="n">
-        <v>67.5407</v>
+        <v>68.94750000000001</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
@@ -3035,7 +3035,7 @@
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:09+00:00</t>
+          <t>2026-07-04T00:36:56+00:00</t>
         </is>
       </c>
     </row>
@@ -3056,22 +3056,22 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>571.1</v>
+        <v>567.7</v>
       </c>
       <c r="E47" t="n">
-        <v>569.6725</v>
+        <v>568.5276</v>
       </c>
       <c r="F47" t="n">
-        <v>36.8617</v>
+        <v>38.1599</v>
       </c>
       <c r="G47" t="n">
-        <v>41.0326</v>
+        <v>39.574</v>
       </c>
       <c r="H47" t="n">
-        <v>37.4112</v>
+        <v>36.9313</v>
       </c>
       <c r="I47" t="n">
-        <v>39.1695</v>
+        <v>38.452</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
@@ -3091,7 +3091,7 @@
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:10+00:00</t>
+          <t>2026-07-04T00:36:56+00:00</t>
         </is>
       </c>
     </row>
@@ -3112,22 +3112,22 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>1457.7</v>
+        <v>1458.2</v>
       </c>
       <c r="E48" t="n">
-        <v>1456.8542</v>
+        <v>1461.4928</v>
       </c>
       <c r="F48" t="n">
-        <v>52.0335</v>
+        <v>50.2488</v>
       </c>
       <c r="G48" t="n">
-        <v>67.01430000000001</v>
+        <v>66.9367</v>
       </c>
       <c r="H48" t="n">
-        <v>59.5992</v>
+        <v>59.6749</v>
       </c>
       <c r="I48" t="n">
-        <v>53.597</v>
+        <v>53.1457</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -3147,7 +3147,7 @@
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:10+00:00</t>
+          <t>2026-07-04T00:36:57+00:00</t>
         </is>
       </c>
     </row>
@@ -3168,22 +3168,22 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>1345.9</v>
+        <v>1374.1</v>
       </c>
       <c r="E49" t="n">
-        <v>1345.4028</v>
+        <v>1375.8233</v>
       </c>
       <c r="F49" t="n">
-        <v>47.344</v>
+        <v>56.676</v>
       </c>
       <c r="G49" t="n">
-        <v>61.8238</v>
+        <v>67.1206</v>
       </c>
       <c r="H49" t="n">
-        <v>59.0799</v>
+        <v>62.3607</v>
       </c>
       <c r="I49" t="n">
-        <v>59.1111</v>
+        <v>60.1251</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
@@ -3203,7 +3203,7 @@
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:11+00:00</t>
+          <t>2026-07-04T00:36:57+00:00</t>
         </is>
       </c>
     </row>
@@ -3224,22 +3224,22 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1140.6</v>
+        <v>1153.4</v>
       </c>
       <c r="E50" t="n">
-        <v>1135.0713</v>
+        <v>1149.4311</v>
       </c>
       <c r="F50" t="n">
-        <v>59.3904</v>
+        <v>61.2102</v>
       </c>
       <c r="G50" t="n">
-        <v>70.3152</v>
+        <v>70.0384</v>
       </c>
       <c r="H50" t="n">
-        <v>61.443</v>
+        <v>62.5233</v>
       </c>
       <c r="I50" t="n">
-        <v>57.531</v>
+        <v>58.5831</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
@@ -3259,7 +3259,7 @@
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:11+00:00</t>
+          <t>2026-07-04T00:36:58+00:00</t>
         </is>
       </c>
     </row>
@@ -3280,22 +3280,22 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>1091.5</v>
+        <v>1116.7</v>
       </c>
       <c r="E51" t="n">
-        <v>1087.213</v>
+        <v>1108.5893</v>
       </c>
       <c r="F51" t="n">
-        <v>47.4407</v>
+        <v>58.7349</v>
       </c>
       <c r="G51" t="n">
-        <v>40.3806</v>
+        <v>48.1616</v>
       </c>
       <c r="H51" t="n">
-        <v>44.7118</v>
+        <v>47.6427</v>
       </c>
       <c r="I51" t="n">
-        <v>50.1532</v>
+        <v>52.72</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
@@ -3315,7 +3315,7 @@
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr">
         <is>
-          <t>2026-07-01T08:18:12+00:00</t>
+          <t>2026-07-04T00:36:59+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>